<commit_message>
Merk fasiten for testeksempel 01 som kontrollert
- Eksepsjonsmeldingene for forfalte frigivelser oppgir nå forfalt antall,
  total frigivelse i uke 1 og tidligste mottaksuke (uke 1 + L).
- Regel 6 presisert, og ny regel 7: forfalt ordremottak vises i uken
  behovet er, selv om det fysisk kommer senere.
- Status i fasit og README endret fra utkast til kontrollert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/testeksempel-01-fasit.xlsx
+++ b/testdata/testeksempel-01-fasit.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Beregningsregler (utkast – gruppen må bekrefte):</t>
+          <t>Beregningsregler (bekreftet av gruppen):</t>
         </is>
       </c>
     </row>
@@ -604,125 +604,110 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>6. Planlagt ordrefrigivelse i uke t − L. Hvis t − L &lt; 1 er frigivelsen forfalt og legges i uke 1 (må frigis straks).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="3" t="inlineStr"/>
+          <t>6. Planlagt ordrefrigivelse i uke t − L. Hvis t − L &lt; 1 er frigivelsen forfalt og legges i uke 1 (må frigis straks), sammen med eventuelle ordinære frigivelser for uke 1. Eksepsjonsmeldingen oppgir hvor mye av uke 1 som er forfalt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>7. Et forfalt planlagt ordremottak vises likevel i uke t, der behovet er, selv om det fysisk kommer tidligst i uke 1 + L. Forventet lagerbeholdning forutsetter altså at behovet dekkes i tide. Avviket varsles med eksepsjonen «Bestilling forsinket» eller «Bruk av sikkerhetslager».</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Eksepsjoner:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>• Bestilling forsinket: frigivelsen er forfalt (t − L &lt; 1) og disponibel(t) &lt; 0. Kunden får ikke levert i tide.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>• Bruk av sikkerhetslager: frigivelsen er forfalt (t − L &lt; 1) og 0 ≤ disponibel(t) &lt; SS. Lageret tærer på sikkerhetslageret før ny leveranse kan komme inn.</t>
+          <t>• Bestilling forsinket: frigivelsen er forfalt (t − L &lt; 1) og disponibel(t) &lt; 0. Kunden får ikke levert i tide.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>• Bruk av sikkerhetslager: frigivelsen er forfalt (t − L &lt; 1) og 0 ≤ disponibel(t) &lt; SS. Lageret tærer på sikkerhetslageret før ny leveranse kan komme inn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>• Mottak forsinket: nettobehov(t) &gt; 0 og det finnes et planlagt mottak i en senere uke. Meldingen peker på første senere mottak, som bør fremskyndes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>• Innkjøpstid overskrider horisont: L ≥ H. Gjelder komponenten (uke «–»), uavhengig av behov.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>• Innkjøpstid overskrider horisont: L ≥ H. Gjelder komponenten (uke «–»), uavhengig av behov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>• En celle kan ha flere eksepsjoner. En komponent med minst én eksepsjon er kritisk.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="3" t="inlineStr"/>
-    </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Status: verdiene er beregnet med skript og MÅ kontrolleres for hånd av gruppen før de brukes som fasit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Status: verdiene er beregnet med skript og kontrollert for hånd (2026-10-19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Hensikt med hver komponent i testeksempelet:</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Komponent-ID</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Navn</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Hensikt</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>K01</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Sete</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Normalforløp: første behov kan bestilles i tide</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>K01</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Rygg</t>
+          <t>Sete</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Normalforløp med innkjøpstid 1 uke</t>
+          <t>Normalforløp: første behov kan bestilles i tide</t>
         </is>
       </c>
       <c r="D24" s="7" t="n"/>
@@ -734,17 +719,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>K02</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Hjul</t>
+          <t>Rygg</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Bestilling forsinket i uke 1 (lager går under 0)</t>
+          <t>Normalforløp med innkjøpstid 1 uke</t>
         </is>
       </c>
       <c r="D25" s="7" t="n"/>
@@ -756,17 +741,17 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>K03</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Armlene</t>
+          <t>Hjul</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Bruk av sikkerhetslager i uke 1 (lager mellom 0 og sikkerhetslager)</t>
+          <t>Bestilling forsinket i uke 1 (lager går under 0)</t>
         </is>
       </c>
       <c r="D26" s="7" t="n"/>
@@ -778,17 +763,17 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>K04</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Gassfjær</t>
+          <t>Armlene</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Mottak forsinket: behov i uke 3, planlagt mottak først i uke 4</t>
+          <t>Bruk av sikkerhetslager i uke 1 (lager mellom 0 og sikkerhetslager)</t>
         </is>
       </c>
       <c r="D27" s="7" t="n"/>
@@ -800,17 +785,17 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>K05</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Stolfot</t>
+          <t>Gassfjær</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Innkjøpstid = horisont (grensetilfelle)</t>
+          <t>Mottak forsinket: behov i uke 3, planlagt mottak først i uke 4</t>
         </is>
       </c>
       <c r="D28" s="7" t="n"/>
@@ -822,17 +807,17 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>K06</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Skruesett</t>
+          <t>Stolfot</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Planlagt mottak i uke 2 kommer i tide (ingen eksepsjon)</t>
+          <t>Innkjøpstid = horisont (grensetilfelle)</t>
         </is>
       </c>
       <c r="D29" s="7" t="n"/>
@@ -844,17 +829,17 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>K07</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Trekk</t>
+          <t>Skruesett</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Sikkerhetslager 0 og frigivelse nøyaktig i uke 1 (grensetilfelle)</t>
+          <t>Planlagt mottak i uke 2 kommer i tide (ingen eksepsjon)</t>
         </is>
       </c>
       <c r="D30" s="7" t="n"/>
@@ -863,17 +848,39 @@
       <c r="G30" s="7" t="n"/>
       <c r="H30" s="8" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>K08</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Trekk</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Sikkerhetslager 0 og frigivelse nøyaktig i uke 1 (grensetilfelle)</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="8" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="26">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="C25:H25"/>
     <mergeCell ref="A15:H15"/>
+    <mergeCell ref="C31:H31"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="C27:H27"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A3:H3"/>
@@ -885,6 +892,7 @@
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C24:H24"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A19:H19"/>
@@ -3054,7 +3062,7 @@
       </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
-          <t>Lager blir -20 i uke 1. Bestillingen måtte vært frigitt i uke 0, før horisonten. Leveranse til kunde blir forsinket.</t>
+          <t>Lager blir -20 i uke 1. Bestillingen på 50 måtte vært frigitt i uke 0, før horisonten. De 50 er forfalt og tatt med i frigivelsen på 175 i uke 1, men kommer tidligst i uke 2. Leveranse til kunde blir forsinket.</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3082,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Lager blir 10 i uke 1, under sikkerhetslager 20, før ny leveranse kan komme inn (måtte vært frigitt i uke 0).</t>
+          <t>Lager blir 10 i uke 1, under sikkerhetslager 20, før ny leveranse kan komme inn. Bestillingen på 10 måtte vært frigitt i uke 0. De 10 er forfalt og tatt med i frigivelsen på 60 i uke 1, men kommer tidligst i uke 2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Testdata: fasit for testeksempel 02 kontrollert for hånd (tall og eksepsjoner)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/testeksempel-01-fasit.xlsx
+++ b/testdata/testeksempel-01-fasit.xlsx
@@ -704,10 +704,10 @@
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="3" t="inlineStr"/>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Status: beregnet med skript, ikke kontrollert for hånd ennå.</t>
+          <t>Status: Kontrollert for hånd av Carmen 2026-10-24 (testeksempel 02, alle 8 deler, tall og eksepsjoner, se testdata/kontroll/). Testeksempel 01 samsvarer med fasiten fra 2026-10-19.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gi MPS-arket nytt navn, forenkle typer og skjerp Kontroll i malen
- «Prognostiserte behov» heter nå «MPS» i malen, README og PRD
- Typer i stykklisten: Ferdigvare, Komponent (Kjøpes inn), Komponent (Produseres selv)
- Ny regel i Veiledning: ikke lim inn i celler med nedtrekksliste
- Kontroll sjekker nivåregelen og ugyldige nivåer og typer
- Testeksempel 01 og fasit laget på nytt med gjeldende mal (tallene er uendret)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/testeksempel-01-fasit.xlsx
+++ b/testdata/testeksempel-01-fasit.xlsx
@@ -562,7 +562,7 @@
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Notasjon: uke t = 1..H, lager før uke 1 = lagerbeholdning, SS = sikkerhetslager, L = innkjøpstid.</t>
+          <t>Notasjon: uke t = 1..H, lager før uke 1 = lagerbeholdning, SS = sikkerhetslager, L = ledetid.</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>• Innkjøpstid overskrider horisont: L ≥ H. Gjelder komponenten (uke «–»), uavhengig av behov.</t>
+          <t>• Ledetid overskrider horisont: L ≥ H. Gjelder komponenten (uke «–»), uavhengig av behov.</t>
         </is>
       </c>
     </row>
@@ -680,12 +680,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Komponent-ID</t>
+          <t>Varenummer</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Navn</t>
+          <t>Beskrivelse</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -697,7 +697,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Normalforløp med innkjøpstid 1 uke</t>
+          <t>Normalforløp med ledetid 1 uke</t>
         </is>
       </c>
       <c r="D25" s="7" t="n"/>
@@ -741,7 +741,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -763,7 +763,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -785,7 +785,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Innkjøpstid = horisont (grensetilfelle)</t>
+          <t>Ledetid = horisont (grensetilfelle)</t>
         </is>
       </c>
       <c r="D29" s="7" t="n"/>
@@ -829,7 +829,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -851,7 +851,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -929,7 +929,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Komponent-ID</t>
+          <t>Varenummer</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -1033,7 +1033,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>300-001</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1243,7 +1243,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1369,7 +1369,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>300-002</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1495,7 +1495,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1537,7 +1537,7 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -1579,7 +1579,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -1663,7 +1663,7 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1705,7 +1705,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -1789,7 +1789,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1831,7 +1831,7 @@
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -1873,7 +1873,7 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1915,7 +1915,7 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -1957,7 +1957,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -2041,7 +2041,7 @@
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -2083,7 +2083,7 @@
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -2125,7 +2125,7 @@
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -2167,7 +2167,7 @@
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -2209,7 +2209,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -2251,7 +2251,7 @@
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -2293,7 +2293,7 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -2335,7 +2335,7 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -2377,7 +2377,7 @@
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -2419,7 +2419,7 @@
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
@@ -2503,7 +2503,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -2545,7 +2545,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -2587,7 +2587,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -2629,7 +2629,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -2671,7 +2671,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -2713,7 +2713,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>K07</t>
+          <t>300-007</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -2755,7 +2755,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -2797,7 +2797,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2839,7 +2839,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2881,7 +2881,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -2923,7 +2923,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -2965,7 +2965,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>K08</t>
+          <t>300-008</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -3027,7 +3027,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Komponent-ID</t>
+          <t>Varenummer</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -3049,7 +3049,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>300-003</t>
         </is>
       </c>
       <c r="B2" s="12" t="n">
@@ -3069,7 +3069,7 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>K04</t>
+          <t>300-004</t>
         </is>
       </c>
       <c r="B3" s="12" t="n">
@@ -3089,7 +3089,7 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>K05</t>
+          <t>300-005</t>
         </is>
       </c>
       <c r="B4" s="12" t="n">
@@ -3109,7 +3109,7 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>K06</t>
+          <t>300-006</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Innkjøpstid overskrider horisont</t>
+          <t>Ledetid overskrider horisont</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Innkjøpstid 10 uker ≥ horisont 10 uker. Ingen ny bestilling kan dekke behov innenfor horisonten.</t>
+          <t>Ledetid 10 uker ≥ horisont 10 uker. Ingen ny bestilling kan dekke behov innenfor horisonten.</t>
         </is>
       </c>
     </row>

</xml_diff>